<commit_message>
Ouvre cinq lignes de construction et cinq d'ameublement dans la projection
Chaque ligne est numerotee, saisie en EUR et convertie en IDR, avec une
colonne de designation libre pour nommer les lots. Deux sous-totaux
alimentent l'investissement total ; les lignes non utilisees comptent pour
zero. Le tableau des revenus previsionnels suit le decalage de lignes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Projection_de_projet.xlsx
+++ b/transactions/Projection_de_projet.xlsx
@@ -179,16 +179,74 @@
         <t>Case a cocher : OUI ajoute les 2 000 EUR de creation de la PT PMA (cellule B12) a l'investissement, NON les retire.</t>
       </text>
     </comment>
-    <comment ref="B35" authorId="0" shapeId="0">
-      <text>
-        <t>Saisir le budget de construction en EUR.
-Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.</t>
-      </text>
-    </comment>
     <comment ref="B36" authorId="0" shapeId="0">
       <text>
-        <t>Saisir le budget d'ameublement en EUR.
-Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.</t>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B37" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B38" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B39" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B40" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B43" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B44" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B45" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B46" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
+      </text>
+    </comment>
+    <comment ref="B47" authorId="0" shapeId="0">
+      <text>
+        <t>Saisir le montant en EUR. Laisser vide si la ligne n'est pas utilisee.
+Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.
+La colonne E permet de nommer la ligne (villa 1, piscine, pool house...).</t>
       </text>
     </comment>
   </commentList>
@@ -484,13 +542,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -820,6 +879,11 @@
           <t>Montant EUR</t>
         </is>
       </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Designation (libre)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -836,26 +900,10 @@
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Cout de construction</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="5">
-        <f>B35*$B$7</f>
-        <v/>
-      </c>
-      <c r="D35" s="3">
-        <f>B35</f>
-        <v/>
-      </c>
-    </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Cout d'ameublement</t>
+          <t>Construction 1</t>
         </is>
       </c>
       <c r="B36" s="3" t="n"/>
@@ -871,13 +919,10 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Creation de la PT PMA (si OUI en B31)</t>
-        </is>
-      </c>
-      <c r="B37" s="3">
-        <f>IF($B$31="OUI",$B$12,0)</f>
-        <v/>
-      </c>
+          <t>Construction 2</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
       <c r="C37" s="5">
         <f>B37*$B$7</f>
         <v/>
@@ -888,249 +933,440 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>INVESTISSEMENT TOTAL</t>
-        </is>
-      </c>
-      <c r="C38" s="6">
-        <f>C34+C35+C36+C37</f>
-        <v/>
-      </c>
-      <c r="D38" s="7">
-        <f>C38/$B$7</f>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Construction 3</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="5">
+        <f>B38*$B$7</f>
+        <v/>
+      </c>
+      <c r="D38" s="3">
+        <f>B38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Construction 4</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="5">
+        <f>B39*$B$7</f>
+        <v/>
+      </c>
+      <c r="D39" s="3">
+        <f>B39</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>3. REVENUS PREVISIONNELS DE LA VILLA</t>
-        </is>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Construction 5</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="5">
+        <f>B40*$B$7</f>
+        <v/>
+      </c>
+      <c r="D40" s="3">
+        <f>B40</f>
+        <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Taux d'occupation previsionnel</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="n">
-        <v>0.65</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Prix moyen de la nuitee (EUR)</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>250</v>
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>SOUS-TOTAL CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="C41" s="6">
+        <f>SUM(C36:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="7">
+        <f>C41/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Nombre de nuits commercialisables / an</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>365</v>
+          <t>Ameublement 1</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="5">
+        <f>B43*$B$7</f>
+        <v/>
+      </c>
+      <c r="D43" s="3">
+        <f>B43</f>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Charges d'exploitation (% du revenu brut)</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="n">
-        <v>0.3</v>
+          <t>Ameublement 2</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="5">
+        <f>B44*$B$7</f>
+        <v/>
+      </c>
+      <c r="D44" s="3">
+        <f>B44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Ameublement 3</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="5">
+        <f>B45*$B$7</f>
+        <v/>
+      </c>
+      <c r="D45" s="3">
+        <f>B45</f>
+        <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>Poste</t>
-        </is>
-      </c>
-      <c r="C46" s="1" t="inlineStr">
-        <is>
-          <t>Montant IDR</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="inlineStr">
-        <is>
-          <t>Montant EUR</t>
-        </is>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Ameublement 4</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="5">
+        <f>B46*$B$7</f>
+        <v/>
+      </c>
+      <c r="D46" s="3">
+        <f>B46</f>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Nuits occupees par an</t>
-        </is>
-      </c>
-      <c r="B47" s="8">
-        <f>B43*B41</f>
+          <t>Ameublement 5</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="5">
+        <f>B47*$B$7</f>
+        <v/>
+      </c>
+      <c r="D47" s="3">
+        <f>B47</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>REVENUS BRUTS ANNUELS</t>
+          <t>SOUS-TOTAL AMEUBLEMENT</t>
         </is>
       </c>
       <c r="C48" s="6">
-        <f>D48*$B$7</f>
+        <f>SUM(C43:C47)</f>
         <v/>
       </c>
       <c r="D48" s="7">
-        <f>B47*$B$42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Charges d'exploitation (30% du revenu brut)</t>
-        </is>
-      </c>
-      <c r="B49" s="4">
-        <f>$B$44</f>
-        <v/>
-      </c>
-      <c r="C49" s="5">
-        <f>C48*$B$44</f>
-        <v/>
-      </c>
-      <c r="D49" s="3">
-        <f>C49/$B$7</f>
+        <f>C48/$B$7</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>REVENUS NETS ANNUELS</t>
-        </is>
-      </c>
-      <c r="C50" s="6">
-        <f>C48-C49</f>
-        <v/>
-      </c>
-      <c r="D50" s="7">
-        <f>C50/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>INDICATEURS</t>
-        </is>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Creation de la PT PMA (si OUI en B31)</t>
+        </is>
+      </c>
+      <c r="B50" s="3">
+        <f>IF($B$31="OUI",$B$12,0)</f>
+        <v/>
+      </c>
+      <c r="C50" s="5">
+        <f>B50*$B$7</f>
+        <v/>
+      </c>
+      <c r="D50" s="3">
+        <f>B50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>INVESTISSEMENT TOTAL</t>
+        </is>
+      </c>
+      <c r="C51" s="6">
+        <f>C34+C41+C48+C50</f>
+        <v/>
+      </c>
+      <c r="D51" s="7">
+        <f>C51/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Rendement brut (revenus bruts / investissement total)</t>
-        </is>
-      </c>
-      <c r="B53" s="4">
-        <f>IF(C38=0,0,C48/C38)</f>
-        <v/>
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>3. REVENUS PREVISIONNELS DE LA VILLA</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Rendement net (revenus nets / investissement total)</t>
-        </is>
-      </c>
-      <c r="B54" s="4">
-        <f>IF(C38=0,0,C50/C38)</f>
-        <v/>
+          <t>Taux d'occupation previsionnel</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="n">
+        <v>0.65</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Retour sur investissement (annees)</t>
-        </is>
-      </c>
-      <c r="B55" s="8">
-        <f>IF(C50=0,0,C38/C50)</f>
-        <v/>
+          <t>Prix moyen de la nuitee (EUR)</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Nombre de nuits commercialisables / an</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>365</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="inlineStr">
-        <is>
-          <t>NOTES / HYPOTHESES</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Tableau 1 : le choix FREEHOLD / LEASEHOLD en B15 pilote le calcul du prix du terrain. Le prix inutilise (B18 ou B19/B20) est simplement ignore.</t>
-        </is>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Charges d'exploitation (% du revenu brut)</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>1 are = 100 m2. Prix freehold exprime en IDR par are ; prix leasehold en IDR par are et par an, multiplie par la duree du bail.</t>
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>Montant IDR</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>Montant EUR</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Frais d'acquisition identiques dans les deux options : taxes gouvernementales 5% (B8) + honoraires du notaire 1% (B9) avec un forfait plancher de 10 000 000 IDR (B10), plus le geometre (B11).</t>
-        </is>
+          <t>Nuits occupees par an</t>
+        </is>
+      </c>
+      <c r="B60" s="8">
+        <f>B56*B54</f>
+        <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Tableau 2 : le cout foncier est repris automatiquement du tableau 1. Construction et ameublement se saisissent en EUR (colonne B) ; pour un devis en IDR, saisir =montant_IDR/$B$7.</t>
-        </is>
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>REVENUS BRUTS ANNUELS</t>
+        </is>
+      </c>
+      <c r="C61" s="6">
+        <f>D61*$B$7</f>
+        <v/>
+      </c>
+      <c r="D61" s="7">
+        <f>B60*$B$55</f>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B31 = OUI.</t>
-        </is>
+          <t>Charges d'exploitation (% du revenu brut)</t>
+        </is>
+      </c>
+      <c r="B62" s="4">
+        <f>$B$57</f>
+        <v/>
+      </c>
+      <c r="C62" s="5">
+        <f>C61*$B$57</f>
+        <v/>
+      </c>
+      <c r="D62" s="3">
+        <f>C62/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Tableau 3 : revenus bruts = nuits commercialisables x taux d'occupation x prix de la nuitee. Les charges sont un pourcentage du revenu brut ; les revenus nets en decoulent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Taux de change en B7 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant presentation au client.</t>
-        </is>
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>REVENUS NETS ANNUELS</t>
+        </is>
+      </c>
+      <c r="C63" s="6">
+        <f>C61-C62</f>
+        <v/>
+      </c>
+      <c r="D63" s="7">
+        <f>C63/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Cellules a saisir : B7 a B12 (parametres), B15 a B20 (terrain), B31 (PT PMA), B35 et B36 (construction et ameublement), B41 a B44 (exploitation). Tout le reste est calcule par formules.</t>
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>INDICATEURS</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Rendement brut (revenus bruts / investissement total)</t>
+        </is>
+      </c>
+      <c r="B66" s="4">
+        <f>IF(C51=0,0,C61/C51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Rendement net (revenus nets / investissement total)</t>
+        </is>
+      </c>
+      <c r="B67" s="4">
+        <f>IF(C51=0,0,C63/C51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Retour sur investissement (annees)</t>
+        </is>
+      </c>
+      <c r="B68" s="8">
+        <f>IF(C63=0,0,C51/C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>NOTES / HYPOTHESES</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Tableau 1 : le choix FREEHOLD / LEASEHOLD en B15 pilote le calcul du prix du terrain. Le prix inutilise (B18 ou B19/B20) est simplement ignore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>1 are = 100 m2. Prix freehold exprime en IDR par are ; prix leasehold en IDR par are et par an, multiplie par la duree du bail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Frais d'acquisition identiques dans les deux options : taxes gouvernementales 5% (B8) + honoraires du notaire 1% (B9) avec un forfait plancher de 10 000 000 IDR (B10), plus le geometre (B11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Tableau 2 : le cout foncier est repris automatiquement du tableau 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Cinq lignes de construction (36 a 40) et cinq lignes d'ameublement (43 a 47) sont disponibles : n'en remplir que le nombre necessaire, les lignes vides comptent pour zero. La colonne E sert a nommer chaque ligne (villa 1, piscine, pool house, lot mobilier...).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Constructions et ameublements se saisissent en EUR (colonne B) ; pour un devis en IDR, saisir =montant_IDR/$B$7. Les sous-totaux des lignes 41 et 48 alimentent l'investissement total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B31 = OUI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Tableau 3 : revenus bruts = nuits commercialisables x taux d'occupation x prix de la nuitee. Les charges sont un pourcentage du revenu brut ; les revenus nets en decoulent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Taux de change en B7 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant presentation au client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Cellules a saisir : B7 a B12 (parametres), B15 a B20 (terrain), B31 (PT PMA), B36 a B47 (constructions et ameublements), B54 a B57 (exploitation). Tout le reste est calcule par formules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>Projection previsionnelle a but indicatif : elle n'integre ni la fiscalite indonesienne sur les revenus locatifs, ni l'amortissement, ni les frais de gestion au-dela du pourcentage de charges saisi.</t>
         </is>

</xml_diff>

<commit_message>
Ajoute emmenagement et ceremonie au cout foncier, et une version client mise en page
Deux nouvelles lignes parametrables dans le tableau du terrain : frais
d'emmenagement et ceremonie traditionnelle, saisis en IDR et repercutes sur le
cout foncier total.

Le meme generateur produit desormais une version destinee au client : la
commission agence y est incorporee au prix du terrain et n'apparait nulle part,
la mise en page est travaillee (bandeaux de section, en-tetes grises,
encadrements, teintes distinctes pour les cellules de saisie et les lignes de
total, montants suffixes IDR et EUR, quadrillage masque) et le bloc de notes
est supprime au profit d'une simple mention indicative. Les libelles des deux
versions sont passes en francais accentue.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Projection_de_projet.xlsx
+++ b/transactions/Projection_de_projet.xlsx
@@ -58,13 +58,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,7 +154,7 @@
   <commentList>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>Taux de reference BCE du 20/08/2026 : 1 EUR = 20 788,62 IDR (source : api.frankfurter.dev). A actualiser au taux du jour.</t>
+        <t>Taux de référence BCE du 20/08/2026 : 1 EUR = 20 788,62 IDR (source : api.frankfurter.dev). À actualiser au taux du jour.</t>
       </text>
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
@@ -163,72 +164,81 @@
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Base annuelle appliquee a toutes les villas (365 nuits, ou moins si la villa est fermee une partie de l'annee).</t>
+        <t>Base annuelle appliquée à toutes les villas (365 nuits, ou moins si la villa est fermée une partie de l'année).</t>
       </text>
     </comment>
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
         <t>Choisir FREEHOLD ou LEASEHOLD dans la liste deroulante.
-FREEHOLD -&gt; prix du terrain = surface x B19 (prix a l'are, sans duree).
-LEASEHOLD -&gt; prix du terrain = surface x B20 x B21 (prix a l'are et par an x duree).</t>
+FREEHOLD -&gt; prix du terrain = surface x B19 (prix à l'are, sans durée).
+LEASEHOLD -&gt; prix du terrain = surface x B20 x B21 (prix à l'are et par an x durée).</t>
       </text>
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
       <text>
-        <t>Case a cocher : OUI ajoute la commission agence (taux de la cellule B23) au prix vendeur, NON la retire.</t>
+        <t>Case à cocher : OUI ajoute la commission agence (taux de la cellule B23) au prix vendeur, NON la retire.</t>
       </text>
     </comment>
     <comment ref="B23" authorId="0" shapeId="0">
       <text>
-        <t>Taux applique au prix vendeur. 25% correspond a un prix vendeur de 4 000 000 IDR/are/an revendu 5 000 000 au client. A ajuster selon le dossier.</t>
+        <t>Taux appliqué au prix vendeur. 25% correspond a un prix vendeur de 4 000 000 IDR/are/an revendu 5 000 000 au client. À ajuster selon le dossier.</t>
       </text>
     </comment>
-    <comment ref="C26" authorId="0" shapeId="0">
+    <comment ref="B24" authorId="0" shapeId="0">
       <text>
-        <t>FREEHOLD : surface x prix a l'are (B17 x B19).
-LEASEHOLD : surface x prix a l'are et par an x duree (B17 x B20 x B21).</t>
+        <t>Montant forfaitaire à renseigner selon le dossier.</t>
+      </text>
+    </comment>
+    <comment ref="B25" authorId="0" shapeId="0">
+      <text>
+        <t>Cérémonie traditionnelle balinaise. Montant forfaitaire a renseigner selon le dossier.</t>
       </text>
     </comment>
     <comment ref="C30" authorId="0" shapeId="0">
       <text>
-        <t>MAX entre le pourcentage d'honoraires (B9) et le forfait minimum (B10) : si le pourcentage donne moins que le forfait, c'est le forfait qui s'applique.
-La colonne Taux affiche le taux reellement supporte.</t>
+        <t>FREEHOLD : surface x prix à l'are.
+LEASEHOLD : surface x prix à l'are et par an x durée.</t>
       </text>
     </comment>
-    <comment ref="B36" authorId="0" shapeId="0">
+    <comment ref="C32" authorId="0" shapeId="0">
       <text>
-        <t>Case a cocher : OUI ajoute les 2 000 EUR de creation de la PT PMA (cellule B12) a l'investissement, NON les retire.</t>
+        <t>MAX entre le pourcentage d'honoraires (B9) et le forfait minimum (B10) : si le pourcentage donne moins que le forfait, c'est le forfait qui s'applique.</t>
       </text>
     </comment>
-    <comment ref="B39" authorId="0" shapeId="0">
+    <comment ref="B40" authorId="0" shapeId="0">
       <text>
-        <t>Nommer chaque villa ici (villa principale, villa 2 chambres, pool house...). La designation est reprise automatiquement dans le tableau des revenus.
-Laisser vide les villas non utilisees : elles comptent pour zero.</t>
+        <t>Case à cocher : OUI ajoute les 2 000 EUR de creation de la PT PMA (cellule B12) a l'investissement, NON les retire.</t>
       </text>
     </comment>
-    <comment ref="C39" authorId="0" shapeId="0">
+    <comment ref="B43" authorId="0" shapeId="0">
       <text>
-        <t>Budget de construction en EUR. Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.</t>
+        <t>Nommer chaque villa ici (villa principale, villa 2 chambres, pool house...). La désignation est reprise automatiquement dans le tableau des revenus.
+Laisser vide les villas non utilisées : elles comptent pour zéro.</t>
       </text>
     </comment>
-    <comment ref="D39" authorId="0" shapeId="0">
+    <comment ref="C43" authorId="0" shapeId="0">
       <text>
-        <t>Budget d'ameublement en EUR. Pour un devis exprime en IDR, saisir la formule =montant_IDR/$B$7.</t>
+        <t>Budget de construction en EUR. Pour un devis exprimé en IDR, saisir la formule =montant_IDR/$B$7.</t>
       </text>
     </comment>
-    <comment ref="B53" authorId="0" shapeId="0">
+    <comment ref="D43" authorId="0" shapeId="0">
       <text>
-        <t>Pourcentage applique au revenu brut cumule de toutes les villas (gestion, menage, entretien, energie...).</t>
+        <t>Budget d'ameublement en EUR. Pour un devis exprimé en IDR, saisir la formule =montant_IDR/$B$7.</t>
       </text>
     </comment>
-    <comment ref="C56" authorId="0" shapeId="0">
+    <comment ref="B57" authorId="0" shapeId="0">
       <text>
-        <t>Taux d'occupation propre a cette villa (ex. 65% = 237 nuits sur 365).</t>
+        <t>Pourcentage appliqué au revenu brut cumulé de toutes les villas (gestion, ménage, entretien, énergie...).</t>
       </text>
     </comment>
-    <comment ref="D56" authorId="0" shapeId="0">
+    <comment ref="C60" authorId="0" shapeId="0">
       <text>
-        <t>Prix moyen de la nuitee de cette villa, en EUR. Laisser vide si la villa n'est pas utilisee dans ce scenario.</t>
+        <t>Taux d'occupation propre à cette villa (ex. 65% = 237 nuits sur 365).</t>
+      </text>
+    </comment>
+    <comment ref="D60" authorId="0" shapeId="0">
+      <text>
+        <t>Prix moyen de la nuitée de cette villa, en EUR. Laisser vide si la villa n'est pas utilisee dans ce scenario.</t>
       </text>
     </comment>
   </commentList>
@@ -524,16 +534,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,6 +559,7 @@
           <t>Client :</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -556,6 +567,7 @@
           <t>Terrain / localisation :</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -563,11 +575,12 @@
           <t>Date :</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>PARAMETRES GENERAUX (cellules a modifier)</t>
+          <t>PARAMÈTRES GÉNÉRAUX</t>
         </is>
       </c>
     </row>
@@ -614,7 +627,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre (EUR)</t>
+          <t>Frais de géomètre (EUR)</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -624,7 +637,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Cout de creation de la PT PMA (EUR)</t>
+          <t>Coût de création de la PT PMA (EUR)</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -644,7 +657,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>1. COUT FONCIER</t>
+          <t>1. COÛT FONCIER</t>
         </is>
       </c>
     </row>
@@ -673,7 +686,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Surface du terrain (m2)</t>
+          <t>Surface du terrain (m²)</t>
         </is>
       </c>
       <c r="B18" s="5">
@@ -702,7 +715,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Duree du leasehold (annees)</t>
+          <t>Durée du leasehold (années)</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -712,7 +725,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Commission agence - a appliquer ? (OUI / NON)</t>
+          <t>Commission agence - à appliquer ? (OUI / NON)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -731,73 +744,60 @@
         <v>0.25</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Frais d'emménagement (IDR)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Cérémonie traditionnelle (IDR)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Taux</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Montant IDR</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>Montant EUR</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Prix du terrain - PRIX VENDEUR</t>
         </is>
       </c>
-      <c r="C26" s="5">
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="5">
         <f>IF($B$16="FREEHOLD",$B$17*$B$19,$B$17*$B$20*$B$21)</f>
         <v/>
       </c>
-      <c r="D26" s="3">
-        <f>C26/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Commission agence (si OUI en B22)</t>
-        </is>
-      </c>
-      <c r="B27" s="4">
-        <f>IF($B$22="OUI",$B$23,0)</f>
-        <v/>
-      </c>
-      <c r="C27" s="5">
-        <f>IF($B$22="OUI",C26*$B$23,0)</f>
-        <v/>
-      </c>
-      <c r="D27" s="3">
-        <f>C27/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>PRIX DU TERRAIN AVEC COMMISSION</t>
-        </is>
-      </c>
-      <c r="C28" s="6">
-        <f>C26+C27</f>
-        <v/>
-      </c>
-      <c r="D28" s="7">
+      <c r="D28" s="3">
         <f>C28/$B$7</f>
         <v/>
       </c>
@@ -805,15 +805,15 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Taxes gouvernementales</t>
+          <t>Commission agence (si OUI en B22)</t>
         </is>
       </c>
       <c r="B29" s="4">
-        <f>$B$8</f>
+        <f>IF($B$22="OUI",$B$23,0)</f>
         <v/>
       </c>
       <c r="C29" s="5">
-        <f>C28*$B$8</f>
+        <f>IF($B$22="OUI",C28*$B$23,0)</f>
         <v/>
       </c>
       <c r="D29" s="3">
@@ -822,20 +822,17 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Honoraires du notaire (forfait plancher en B10)</t>
-        </is>
-      </c>
-      <c r="B30" s="4">
-        <f>IF(C28=0,0,C30/C28)</f>
-        <v/>
-      </c>
-      <c r="C30" s="5">
-        <f>MAX(C28*$B$9,$B$10)</f>
-        <v/>
-      </c>
-      <c r="D30" s="3">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>PRIX DU TERRAIN AVEC COMMISSION</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="7">
+        <f>C28+C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="8">
         <f>C30/$B$7</f>
         <v/>
       </c>
@@ -843,15 +840,15 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+          <t>Taxes gouvernementales</t>
         </is>
       </c>
       <c r="B31" s="4">
-        <f>IF(C28=0,0,C31/C28)</f>
+        <f>$B$8</f>
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>C29+C30</f>
+        <f>C30*$B$8</f>
         <v/>
       </c>
       <c r="D31" s="3">
@@ -862,162 +859,163 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Frais de geometre (forfait)</t>
-        </is>
+          <t>Honoraires du notaire (forfait plancher en B10)</t>
+        </is>
+      </c>
+      <c r="B32" s="4">
+        <f>IF(C30=0,0,C32/C30)</f>
+        <v/>
       </c>
       <c r="C32" s="5">
+        <f>MAX(C30*$B$9,$B$10)</f>
+        <v/>
+      </c>
+      <c r="D32" s="3">
+        <f>C32/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Sous-total frais de notaire (taxes + honoraires)</t>
+        </is>
+      </c>
+      <c r="B33" s="4">
+        <f>IF(C30=0,0,C33/C30)</f>
+        <v/>
+      </c>
+      <c r="C33" s="5">
+        <f>C31+C32</f>
+        <v/>
+      </c>
+      <c r="D33" s="3">
+        <f>C33/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Frais de géomètre (forfait)</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="5">
         <f>$B$11*$B$7</f>
         <v/>
       </c>
-      <c r="D32" s="3">
+      <c r="D34" s="3">
         <f>$B$11</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>COUT FONCIER TOTAL</t>
-        </is>
-      </c>
-      <c r="C33" s="6">
-        <f>C28+C31+C32</f>
-        <v/>
-      </c>
-      <c r="D33" s="7">
-        <f>C33/$B$7</f>
-        <v/>
-      </c>
-    </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>2. INVESTISSEMENT A CONSENTIR</t>
-        </is>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Frais d'emménagement</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="5">
+        <f>$B$24</f>
+        <v/>
+      </c>
+      <c r="D35" s="3">
+        <f>C35/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Creation de la PT PMA - a inclure ? (OUI / NON)</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>OUI</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="1" t="inlineStr">
-        <is>
-          <t>Designation de la villa</t>
-        </is>
-      </c>
-      <c r="C38" s="1" t="inlineStr">
-        <is>
-          <t>Construction (EUR)</t>
-        </is>
-      </c>
-      <c r="D38" s="1" t="inlineStr">
-        <is>
-          <t>Ameublement (EUR)</t>
-        </is>
-      </c>
-      <c r="E38" s="1" t="inlineStr">
-        <is>
-          <t>Total villa (EUR)</t>
-        </is>
-      </c>
-      <c r="F38" s="1" t="inlineStr">
-        <is>
-          <t>Total villa (IDR)</t>
-        </is>
+          <t>Cérémonie traditionnelle</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="5">
+        <f>$B$25</f>
+        <v/>
+      </c>
+      <c r="D36" s="3">
+        <f>C36/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>COÛT FONCIER TOTAL</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="7">
+        <f>C30+C33+C34+C35+C36</f>
+        <v/>
+      </c>
+      <c r="D37" s="8">
+        <f>C37/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>Villa 1</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Villa 1</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3">
-        <f>C39+D39</f>
-        <v/>
-      </c>
-      <c r="F39" s="5">
-        <f>E39*$B$7</f>
-        <v/>
+          <t>2. INVESTISSEMENT À CONSENTIR</t>
+        </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>Villa 2</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3">
-        <f>C40+D40</f>
-        <v/>
-      </c>
-      <c r="F40" s="5">
-        <f>E40*$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>Villa 3</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3">
-        <f>C41+D41</f>
-        <v/>
-      </c>
-      <c r="F41" s="5">
-        <f>E41*$B$7</f>
-        <v/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Création de la PT PMA - à inclure ? (OUI / NON)</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t>Villa 4</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3">
-        <f>C42+D42</f>
-        <v/>
-      </c>
-      <c r="F42" s="5">
-        <f>E42*$B$7</f>
-        <v/>
+      <c r="A42" s="1" t="inlineStr"/>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>Désignation de la villa</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>Construction (EUR)</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>Ameublement (EUR)</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Total villa (EUR)</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>Total villa (IDR)</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>Villa 5</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="n"/>
+          <t>Villa 1</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Villa 1</t>
+        </is>
+      </c>
       <c r="C43" s="3" t="n"/>
       <c r="D43" s="3" t="n"/>
       <c r="E43" s="3">
@@ -1032,269 +1030,252 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>TOTAL VILLAS</t>
-        </is>
-      </c>
-      <c r="C44" s="7">
-        <f>SUM(C39:C43)</f>
-        <v/>
-      </c>
-      <c r="D44" s="7">
-        <f>SUM(D39:D43)</f>
-        <v/>
-      </c>
-      <c r="E44" s="7">
-        <f>SUM(E39:E43)</f>
-        <v/>
-      </c>
-      <c r="F44" s="6">
+          <t>Villa 2</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3">
+        <f>C44+D44</f>
+        <v/>
+      </c>
+      <c r="F44" s="5">
         <f>E44*$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Villa 3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3">
+        <f>C45+D45</f>
+        <v/>
+      </c>
+      <c r="F45" s="5">
+        <f>E45*$B$7</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>Poste</t>
-        </is>
-      </c>
-      <c r="C46" s="1" t="inlineStr">
-        <is>
-          <t>Montant IDR</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="inlineStr">
-        <is>
-          <t>Montant EUR</t>
-        </is>
+          <t>Villa 4</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3">
+        <f>C46+D46</f>
+        <v/>
+      </c>
+      <c r="F46" s="5">
+        <f>E46*$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Cout foncier (report du tableau 1)</t>
-        </is>
-      </c>
-      <c r="C47" s="5">
-        <f>C33</f>
-        <v/>
-      </c>
-      <c r="D47" s="3">
-        <f>C47/$B$7</f>
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>Villa 5</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="3" t="n"/>
+      <c r="E47" s="3">
+        <f>C47+D47</f>
+        <v/>
+      </c>
+      <c r="F47" s="5">
+        <f>E47*$B$7</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Constructions et ameublements (total villas)</t>
-        </is>
-      </c>
-      <c r="C48" s="5">
-        <f>F44</f>
-        <v/>
-      </c>
-      <c r="D48" s="3">
-        <f>C48/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Creation de la PT PMA (si OUI en B36)</t>
-        </is>
-      </c>
-      <c r="C49" s="5">
-        <f>IF($B$36="OUI",$B$12*$B$7,0)</f>
-        <v/>
-      </c>
-      <c r="D49" s="3">
-        <f>C49/$B$7</f>
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL VILLAS</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="8">
+        <f>SUM(C43:C47)</f>
+        <v/>
+      </c>
+      <c r="D48" s="8">
+        <f>SUM(D43:D47)</f>
+        <v/>
+      </c>
+      <c r="E48" s="8">
+        <f>SUM(E43:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="7">
+        <f>E48*$B$7</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>INVESTISSEMENT TOTAL</t>
-        </is>
-      </c>
-      <c r="C50" s="6">
-        <f>C47+C48+C49</f>
-        <v/>
-      </c>
-      <c r="D50" s="7">
-        <f>C50/$B$7</f>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>Taux</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>Montant IDR</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>Montant EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Coût foncier (report du tableau 1)</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="5">
+        <f>C37</f>
+        <v/>
+      </c>
+      <c r="D51" s="3">
+        <f>C51/$B$7</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>3. REVENUS PREVISIONNELS PAR VILLA</t>
-        </is>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Constructions et ameublements (total villas)</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="5">
+        <f>F48</f>
+        <v/>
+      </c>
+      <c r="D52" s="3">
+        <f>C52/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Charges d'exploitation (% du revenu brut)</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>Designation de la villa</t>
-        </is>
-      </c>
-      <c r="C55" s="1" t="inlineStr">
-        <is>
-          <t>Taux d'occupation</t>
-        </is>
-      </c>
-      <c r="D55" s="1" t="inlineStr">
-        <is>
-          <t>Prix nuitee (EUR)</t>
-        </is>
-      </c>
-      <c r="E55" s="1" t="inlineStr">
-        <is>
-          <t>Nuits occupees / an</t>
-        </is>
-      </c>
-      <c r="F55" s="1" t="inlineStr">
-        <is>
-          <t>Revenus bruts (EUR)</t>
-        </is>
-      </c>
-      <c r="G55" s="1" t="inlineStr">
-        <is>
-          <t>Revenus bruts (IDR)</t>
-        </is>
+          <t>Création de la PT PMA (si OUI en B40)</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="5">
+        <f>IF($B$40="OUI",$B$12*$B$7,0)</f>
+        <v/>
+      </c>
+      <c r="D53" s="3">
+        <f>C53/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>INVESTISSEMENT TOTAL</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="7">
+        <f>C51+C52+C53</f>
+        <v/>
+      </c>
+      <c r="D54" s="8">
+        <f>C54/$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>Villa 1</t>
-        </is>
-      </c>
-      <c r="B56" s="2">
-        <f>IF($B$39="","",$B$39)</f>
-        <v/>
-      </c>
-      <c r="C56" s="4" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D56" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="E56" s="8">
-        <f>$B$13*C56</f>
-        <v/>
-      </c>
-      <c r="F56" s="3">
-        <f>E56*D56</f>
-        <v/>
-      </c>
-      <c r="G56" s="5">
-        <f>F56*$B$7</f>
-        <v/>
+          <t>3. REVENUS PRÉVISIONNELS PAR VILLA</t>
+        </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="inlineStr">
-        <is>
-          <t>Villa 2</t>
-        </is>
-      </c>
-      <c r="B57" s="2">
-        <f>IF($B$40="","",$B$40)</f>
-        <v/>
-      </c>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="3" t="n"/>
-      <c r="E57" s="8">
-        <f>$B$13*C57</f>
-        <v/>
-      </c>
-      <c r="F57" s="3">
-        <f>E57*D57</f>
-        <v/>
-      </c>
-      <c r="G57" s="5">
-        <f>F57*$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="inlineStr">
-        <is>
-          <t>Villa 3</t>
-        </is>
-      </c>
-      <c r="B58" s="2">
-        <f>IF($B$41="","",$B$41)</f>
-        <v/>
-      </c>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="8">
-        <f>$B$13*C58</f>
-        <v/>
-      </c>
-      <c r="F58" s="3">
-        <f>E58*D58</f>
-        <v/>
-      </c>
-      <c r="G58" s="5">
-        <f>F58*$B$7</f>
-        <v/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Charges d'exploitation (% du revenu brut)</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t>Villa 4</t>
-        </is>
-      </c>
-      <c r="B59" s="2">
-        <f>IF($B$42="","",$B$42)</f>
-        <v/>
-      </c>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="3" t="n"/>
-      <c r="E59" s="8">
-        <f>$B$13*C59</f>
-        <v/>
-      </c>
-      <c r="F59" s="3">
-        <f>E59*D59</f>
-        <v/>
-      </c>
-      <c r="G59" s="5">
-        <f>F59*$B$7</f>
-        <v/>
+      <c r="A59" s="1" t="inlineStr"/>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>Désignation de la villa</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>Taux d'occupation</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>Prix nuitée (EUR)</t>
+        </is>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>Nuits occupées / an</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>Revenus bruts (EUR)</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="inlineStr">
+        <is>
+          <t>Revenus bruts (IDR)</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>Villa 5</t>
+          <t>Villa 1</t>
         </is>
       </c>
       <c r="B60" s="2">
         <f>IF($B$43="","",$B$43)</f>
         <v/>
       </c>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="3" t="n"/>
-      <c r="E60" s="8">
+      <c r="C60" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="E60" s="9">
         <f>$B$13*C60</f>
         <v/>
       </c>
@@ -1310,218 +1291,330 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
+          <t>Villa 2</t>
+        </is>
+      </c>
+      <c r="B61" s="2">
+        <f>IF($B$44="","",$B$44)</f>
+        <v/>
+      </c>
+      <c r="C61" s="4" t="n"/>
+      <c r="D61" s="3" t="n"/>
       <c r="E61" s="9">
-        <f>SUM(E56:E60)</f>
-        <v/>
-      </c>
-      <c r="F61" s="7">
-        <f>SUM(F56:F60)</f>
-        <v/>
-      </c>
-      <c r="G61" s="6">
-        <f>SUM(G56:G60)</f>
+        <f>$B$13*C61</f>
+        <v/>
+      </c>
+      <c r="F61" s="3">
+        <f>E61*D61</f>
+        <v/>
+      </c>
+      <c r="G61" s="5">
+        <f>F61*$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>Villa 3</t>
+        </is>
+      </c>
+      <c r="B62" s="2">
+        <f>IF($B$45="","",$B$45)</f>
+        <v/>
+      </c>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="9">
+        <f>$B$13*C62</f>
+        <v/>
+      </c>
+      <c r="F62" s="3">
+        <f>E62*D62</f>
+        <v/>
+      </c>
+      <c r="G62" s="5">
+        <f>F62*$B$7</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>Poste</t>
-        </is>
-      </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t>Taux</t>
-        </is>
-      </c>
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t>Montant IDR</t>
-        </is>
-      </c>
-      <c r="D63" s="1" t="inlineStr">
-        <is>
-          <t>Montant EUR</t>
-        </is>
+          <t>Villa 4</t>
+        </is>
+      </c>
+      <c r="B63" s="2">
+        <f>IF($B$46="","",$B$46)</f>
+        <v/>
+      </c>
+      <c r="C63" s="4" t="n"/>
+      <c r="D63" s="3" t="n"/>
+      <c r="E63" s="9">
+        <f>$B$13*C63</f>
+        <v/>
+      </c>
+      <c r="F63" s="3">
+        <f>E63*D63</f>
+        <v/>
+      </c>
+      <c r="G63" s="5">
+        <f>F63*$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>REVENUS BRUTS ANNUELS</t>
-        </is>
-      </c>
-      <c r="C64" s="6">
-        <f>G61</f>
-        <v/>
-      </c>
-      <c r="D64" s="7">
-        <f>F61</f>
+          <t>Villa 5</t>
+        </is>
+      </c>
+      <c r="B64" s="2">
+        <f>IF($B$47="","",$B$47)</f>
+        <v/>
+      </c>
+      <c r="C64" s="4" t="n"/>
+      <c r="D64" s="3" t="n"/>
+      <c r="E64" s="9">
+        <f>$B$13*C64</f>
+        <v/>
+      </c>
+      <c r="F64" s="3">
+        <f>E64*D64</f>
+        <v/>
+      </c>
+      <c r="G64" s="5">
+        <f>F64*$B$7</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Charges d'exploitation</t>
-        </is>
-      </c>
-      <c r="B65" s="4">
-        <f>$B$53</f>
-        <v/>
-      </c>
-      <c r="C65" s="5">
-        <f>C64*$B$53</f>
-        <v/>
-      </c>
-      <c r="D65" s="3">
-        <f>C65/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="inlineStr">
-        <is>
-          <t>REVENUS NETS ANNUELS</t>
-        </is>
-      </c>
-      <c r="C66" s="6">
-        <f>C64-C65</f>
-        <v/>
-      </c>
-      <c r="D66" s="7">
-        <f>C66/$B$7</f>
-        <v/>
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="10">
+        <f>SUM(E60:E64)</f>
+        <v/>
+      </c>
+      <c r="F65" s="8">
+        <f>SUM(F60:F64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="7">
+        <f>SUM(G60:G64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>Taux</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr">
+        <is>
+          <t>Montant IDR</t>
+        </is>
+      </c>
+      <c r="D67" s="1" t="inlineStr">
+        <is>
+          <t>Montant EUR</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>INDICATEURS</t>
-        </is>
+          <t>REVENUS BRUTS ANNUELS</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="7">
+        <f>G65</f>
+        <v/>
+      </c>
+      <c r="D68" s="8">
+        <f>F65</f>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Nombre de villas retenues dans le scenario</t>
-        </is>
-      </c>
-      <c r="B69" s="5">
-        <f>COUNTIF(D56:D60,"&gt;0")</f>
+          <t>Charges d'exploitation</t>
+        </is>
+      </c>
+      <c r="B69" s="4">
+        <f>$B$57</f>
+        <v/>
+      </c>
+      <c r="C69" s="5">
+        <f>C68*$B$57</f>
+        <v/>
+      </c>
+      <c r="D69" s="3">
+        <f>C69/$B$7</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>REVENUS NETS ANNUELS</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="7">
+        <f>C68-C69</f>
+        <v/>
+      </c>
+      <c r="D70" s="8">
+        <f>C70/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>INDICATEURS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Nombre de villas retenues dans le scénario</t>
+        </is>
+      </c>
+      <c r="B73" s="7">
+        <f>COUNTIF(D60:D64,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>Rendement brut (revenus bruts / investissement total)</t>
         </is>
       </c>
-      <c r="B70" s="4">
-        <f>IF(C50=0,0,C64/C50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Rendement net (revenus nets / investissement total)</t>
-        </is>
-      </c>
-      <c r="B71" s="4">
-        <f>IF(C50=0,0,C66/C50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Retour sur investissement (annees)</t>
-        </is>
-      </c>
-      <c r="B72" s="8">
-        <f>IF(C66=0,0,C50/C66)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="1" t="inlineStr">
-        <is>
-          <t>NOTES / HYPOTHESES</t>
-        </is>
+      <c r="B74" s="6">
+        <f>IF(C54=0,0,C68/C54)</f>
+        <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>MODE D'EMPLOI : renseigner le terrain (tableau 1), nommer les villas et saisir leurs budgets (tableau 2), puis leur occupation et leur prix de nuitee (tableau 3). Les villas non utilisees restent vides et comptent pour zero.</t>
-        </is>
+          <t>Rendement net (revenus nets / investissement total)</t>
+        </is>
+      </c>
+      <c r="B75" s="6">
+        <f>IF(C54=0,0,C70/C54)</f>
+        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Tableau 1 : le choix FREEHOLD / LEASEHOLD en B16 pilote le calcul du prix du terrain ; le prix inutilise (B19 ou B20/B21) est simplement ignore. 1 are = 100 m2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Les prix du terrain sont des PRIX VENDEUR : la commission agence est ajoutee separement en ligne 27, uniquement si B22 = OUI, au taux de la cellule B23.</t>
-        </is>
+          <t>Retour sur investissement (années)</t>
+        </is>
+      </c>
+      <c r="B76" s="10">
+        <f>IF(C70=0,0,C54/C70)</f>
+        <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 28) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10). S'y ajoute le geometre (B11).</t>
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>NOTES / HYPOTHESES</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Tableau 2 : une ligne par villa, construction et ameublement saisis en EUR ; pour un devis en IDR, saisir =montant_IDR/$B$7. La designation saisie en colonne B est reprise automatiquement dans le tableau 3.</t>
+          <t>MODE D'EMPLOI : renseigner le terrain (tableau 1), nommer les villas et saisir leurs budgets (tableau 2), puis leur occupation et leur prix de nuitee (tableau 3). Les villas non utilisees restent vides et comptent pour zero.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B36 = OUI. Elle est unique pour le projet, quel que soit le nombre de villas.</t>
+          <t>Tableau 1 : le choix FREEHOLD / LEASEHOLD en B16 pilote le calcul du prix du terrain ; le prix inutilise est simplement ignore. 1 are = 100 m2.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Tableau 3 : chaque villa a son propre taux d'occupation et son propre prix de nuitee. Revenus bruts d'une villa = nuits commercialisables (B13) x taux d'occupation x prix de la nuitee. Les charges s'appliquent au revenu brut cumule.</t>
+          <t>Les prix du terrain sont des PRIX VENDEUR : la commission agence est ajoutee separement en ligne 29, uniquement si B22 = OUI, au taux de la cellule B23.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Taux de change en B7 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant presentation au client.</t>
+          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 30) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Toutes les cellules a saisir sont en colonne B (parametres et options) et dans les colonnes B, C et D des deux grilles villas. Tout le reste est calcule par formules.</t>
+          <t>S'ajoutent au cout foncier le geometre (B11), les frais d'emmenagement (B24) et la ceremonie traditionnelle (B25), saisis en IDR.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
+          <t>Tableau 2 : une ligne par villa, construction et ameublement saisis en EUR ; pour un devis en IDR, saisir =montant_IDR/$B$7. La designation saisie en colonne B est reprise automatiquement dans le tableau 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B40 = OUI, quel que soit le nombre de villas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Tableau 3 : chaque villa a son propre taux d'occupation et son propre prix de nuitee. Revenus bruts = nuits commercialisables (B13) x taux d'occupation x prix de la nuitee. Les charges s'appliquent au revenu brut cumule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Taux de change en B7 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant presentation au client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
           <t>Projection previsionnelle a but indicatif : elle n'integre ni la fiscalite indonesienne sur les revenus locatifs, ni l'amortissement, ni les frais de gestion au-dela du pourcentage de charges saisi. En leasehold, le rendement doit s'apprecier au regard de la duree residuelle du bail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="inlineStr">
+        <is>
+          <t>VERSION INTERNE - contient la commission agence. Ne pas transmettre au client : utiliser la version 'presentation client'.</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1626,7 @@
     <dataValidation sqref="B22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"OUI,NON"</formula1>
     </dataValidation>
-    <dataValidation sqref="B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"OUI,NON"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Neutralise visuellement les cellules sans objet selon l'option foncière
En FREEHOLD, la durée du leasehold et le prix à l'are et par an sont grisés
par mise en forme conditionnelle et portent la mention 'sans objet en
FREEHOLD' ; en LEASEHOLD c'est le prix freehold qui l'est. La cellule de prix
réellement attendue par l'option retenue affiche 'A RENSEIGNER' tant qu'elle
est vide, ce qui rend visible la seule saisie qui bloque le calcul.

La durée n'a jamais été utilisée hors de la branche LEASEHOLD de la formule :
le calcul freehold aboutit qu'elle soit remplie, vidée ou textuelle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Projection_de_projet.xlsx
+++ b/transactions/Projection_de_projet.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,12 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -58,13 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -74,6 +81,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <i val="1"/>
+        <color rgb="00A6A6A6"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00F2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -172,6 +192,11 @@
         <t>Choisir FREEHOLD ou LEASEHOLD dans la liste deroulante.
 FREEHOLD -&gt; prix du terrain = surface x B19 (prix à l'are, sans durée).
 LEASEHOLD -&gt; prix du terrain = surface x B20 x B21 (prix à l'are et par an x durée).</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0">
+      <text>
+        <t>Utilisee uniquement en LEASEHOLD. En FREEHOLD la cellule est grisee et n'entre dans aucun calcul.</t>
       </text>
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
@@ -701,6 +726,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6">
+        <f>IF($B$16="FREEHOLD",IF($B$19&gt;0,"","A RENSEIGNER"),"sans objet en LEASEHOLD")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -711,6 +740,10 @@
       <c r="B20" s="5" t="n">
         <v>4000000</v>
       </c>
+      <c r="C20" s="6">
+        <f>IF($B$16="LEASEHOLD",IF($B$20&gt;0,"","A RENSEIGNER"),"sans objet en FREEHOLD")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -720,6 +753,10 @@
       </c>
       <c r="B21" s="5" t="n">
         <v>30</v>
+      </c>
+      <c r="C21" s="6">
+        <f>IF($B$16="LEASEHOLD",IF($B$21&gt;0,"","A RENSEIGNER"),"sans objet en FREEHOLD")</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -827,12 +864,12 @@
           <t>PRIX DU TERRAIN AVEC COMMISSION</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="7">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="8">
         <f>C28+C29</f>
         <v/>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="9">
         <f>C30/$B$7</f>
         <v/>
       </c>
@@ -948,12 +985,12 @@
           <t>COÛT FONCIER TOTAL</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="7">
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="8">
         <f>C30+C33+C34+C35+C36</f>
         <v/>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="9">
         <f>C37/$B$7</f>
         <v/>
       </c>
@@ -1106,19 +1143,19 @@
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
-      <c r="C48" s="8">
+      <c r="C48" s="9">
         <f>SUM(C43:C47)</f>
         <v/>
       </c>
-      <c r="D48" s="8">
+      <c r="D48" s="9">
         <f>SUM(D43:D47)</f>
         <v/>
       </c>
-      <c r="E48" s="8">
+      <c r="E48" s="9">
         <f>SUM(E43:E47)</f>
         <v/>
       </c>
-      <c r="F48" s="7">
+      <c r="F48" s="8">
         <f>E48*$B$7</f>
         <v/>
       </c>
@@ -1199,12 +1236,12 @@
           <t>INVESTISSEMENT TOTAL</t>
         </is>
       </c>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="7">
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="8">
         <f>C51+C52+C53</f>
         <v/>
       </c>
-      <c r="D54" s="8">
+      <c r="D54" s="9">
         <f>C54/$B$7</f>
         <v/>
       </c>
@@ -1275,7 +1312,7 @@
       <c r="D60" s="3" t="n">
         <v>250</v>
       </c>
-      <c r="E60" s="9">
+      <c r="E60" s="10">
         <f>$B$13*C60</f>
         <v/>
       </c>
@@ -1300,7 +1337,7 @@
       </c>
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="3" t="n"/>
-      <c r="E61" s="9">
+      <c r="E61" s="10">
         <f>$B$13*C61</f>
         <v/>
       </c>
@@ -1325,7 +1362,7 @@
       </c>
       <c r="C62" s="4" t="n"/>
       <c r="D62" s="3" t="n"/>
-      <c r="E62" s="9">
+      <c r="E62" s="10">
         <f>$B$13*C62</f>
         <v/>
       </c>
@@ -1350,7 +1387,7 @@
       </c>
       <c r="C63" s="4" t="n"/>
       <c r="D63" s="3" t="n"/>
-      <c r="E63" s="9">
+      <c r="E63" s="10">
         <f>$B$13*C63</f>
         <v/>
       </c>
@@ -1375,7 +1412,7 @@
       </c>
       <c r="C64" s="4" t="n"/>
       <c r="D64" s="3" t="n"/>
-      <c r="E64" s="9">
+      <c r="E64" s="10">
         <f>$B$13*C64</f>
         <v/>
       </c>
@@ -1397,15 +1434,15 @@
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n"/>
-      <c r="E65" s="10">
+      <c r="E65" s="11">
         <f>SUM(E60:E64)</f>
         <v/>
       </c>
-      <c r="F65" s="8">
+      <c r="F65" s="9">
         <f>SUM(F60:F64)</f>
         <v/>
       </c>
-      <c r="G65" s="7">
+      <c r="G65" s="8">
         <f>SUM(G60:G64)</f>
         <v/>
       </c>
@@ -1439,11 +1476,11 @@
         </is>
       </c>
       <c r="B68" s="2" t="n"/>
-      <c r="C68" s="7">
+      <c r="C68" s="8">
         <f>G65</f>
         <v/>
       </c>
-      <c r="D68" s="8">
+      <c r="D68" s="9">
         <f>F65</f>
         <v/>
       </c>
@@ -1473,12 +1510,12 @@
           <t>REVENUS NETS ANNUELS</t>
         </is>
       </c>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="7">
+      <c r="B70" s="7" t="n"/>
+      <c r="C70" s="8">
         <f>C68-C69</f>
         <v/>
       </c>
-      <c r="D70" s="8">
+      <c r="D70" s="9">
         <f>C70/$B$7</f>
         <v/>
       </c>
@@ -1496,7 +1533,7 @@
           <t>Nombre de villas retenues dans le scénario</t>
         </is>
       </c>
-      <c r="B73" s="7">
+      <c r="B73" s="8">
         <f>COUNTIF(D60:D64,"&gt;0")</f>
         <v/>
       </c>
@@ -1507,7 +1544,7 @@
           <t>Rendement brut (revenus bruts / investissement total)</t>
         </is>
       </c>
-      <c r="B74" s="6">
+      <c r="B74" s="7">
         <f>IF(C54=0,0,C68/C54)</f>
         <v/>
       </c>
@@ -1518,7 +1555,7 @@
           <t>Rendement net (revenus nets / investissement total)</t>
         </is>
       </c>
-      <c r="B75" s="6">
+      <c r="B75" s="7">
         <f>IF(C54=0,0,C70/C54)</f>
         <v/>
       </c>
@@ -1529,7 +1566,7 @@
           <t>Retour sur investissement (années)</t>
         </is>
       </c>
-      <c r="B76" s="10">
+      <c r="B76" s="11">
         <f>IF(C70=0,0,C54/C70)</f>
         <v/>
       </c>
@@ -1619,6 +1656,21 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A19:C19">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$B$16&lt;&gt;"FREEHOLD"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20:C20">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$B$16&lt;&gt;"LEASEHOLD"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A21:C21">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$B$16&lt;&gt;"LEASEHOLD"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"FREEHOLD,LEASEHOLD"</formula1>

</xml_diff>

<commit_message>
Ajoute l'impôt sur les sociétés de 0,5% du chiffre d'affaires aux charges
Nouveau taux paramétrable dans le tableau des revenus, applique au revenu
brut cumulé. Le bloc des charges distingue désormais charges d'exploitation,
impôt sur les sociétés et total des charges, dont découlent les revenus nets
et les indicateurs de rendement.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Projection_de_projet.xlsx
+++ b/transactions/Projection_de_projet.xlsx
@@ -256,12 +256,17 @@
         <t>Pourcentage appliqué au revenu brut cumulé de toutes les villas (gestion, ménage, entretien, énergie...).</t>
       </text>
     </comment>
-    <comment ref="C60" authorId="0" shapeId="0">
+    <comment ref="B58" authorId="0" shapeId="0">
+      <text>
+        <t>Impôt assis sur le chiffre d'affaires brut, et non sur le résultat : il est dû même si l'exploitation ne dégage pas de bénéfice.</t>
+      </text>
+    </comment>
+    <comment ref="C61" authorId="0" shapeId="0">
       <text>
         <t>Taux d'occupation propre à cette villa (ex. 65% = 237 nuits sur 365).</t>
       </text>
     </comment>
-    <comment ref="D60" authorId="0" shapeId="0">
+    <comment ref="D61" authorId="0" shapeId="0">
       <text>
         <t>Prix moyen de la nuitée de cette villa, en EUR. Laisser vide si la villa n'est pas utilisee dans ce scenario.</t>
       </text>
@@ -559,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1263,80 +1268,65 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="1" t="inlineStr"/>
-      <c r="B59" s="1" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Impôt sur les sociétés (% du chiffre d'affaires)</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr"/>
+      <c r="B60" s="1" t="inlineStr">
         <is>
           <t>Désignation de la villa</t>
         </is>
       </c>
-      <c r="C59" s="1" t="inlineStr">
+      <c r="C60" s="1" t="inlineStr">
         <is>
           <t>Taux d'occupation</t>
         </is>
       </c>
-      <c r="D59" s="1" t="inlineStr">
+      <c r="D60" s="1" t="inlineStr">
         <is>
           <t>Prix nuitée (EUR)</t>
         </is>
       </c>
-      <c r="E59" s="1" t="inlineStr">
+      <c r="E60" s="1" t="inlineStr">
         <is>
           <t>Nuits occupées / an</t>
         </is>
       </c>
-      <c r="F59" s="1" t="inlineStr">
+      <c r="F60" s="1" t="inlineStr">
         <is>
           <t>Revenus bruts (EUR)</t>
         </is>
       </c>
-      <c r="G59" s="1" t="inlineStr">
+      <c r="G60" s="1" t="inlineStr">
         <is>
           <t>Revenus bruts (IDR)</t>
         </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>Villa 1</t>
-        </is>
-      </c>
-      <c r="B60" s="2">
-        <f>IF($B$43="","",$B$43)</f>
-        <v/>
-      </c>
-      <c r="C60" s="4" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="E60" s="10">
-        <f>$B$13*C60</f>
-        <v/>
-      </c>
-      <c r="F60" s="3">
-        <f>E60*D60</f>
-        <v/>
-      </c>
-      <c r="G60" s="5">
-        <f>F60*$B$7</f>
-        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>Villa 2</t>
+          <t>Villa 1</t>
         </is>
       </c>
       <c r="B61" s="2">
-        <f>IF($B$44="","",$B$44)</f>
-        <v/>
-      </c>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="3" t="n"/>
+        <f>IF($B$43="","",$B$43)</f>
+        <v/>
+      </c>
+      <c r="C61" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>250</v>
+      </c>
       <c r="E61" s="10">
         <f>$B$13*C61</f>
         <v/>
@@ -1353,11 +1343,11 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>Villa 3</t>
+          <t>Villa 2</t>
         </is>
       </c>
       <c r="B62" s="2">
-        <f>IF($B$45="","",$B$45)</f>
+        <f>IF($B$44="","",$B$44)</f>
         <v/>
       </c>
       <c r="C62" s="4" t="n"/>
@@ -1378,11 +1368,11 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>Villa 4</t>
+          <t>Villa 3</t>
         </is>
       </c>
       <c r="B63" s="2">
-        <f>IF($B$46="","",$B$46)</f>
+        <f>IF($B$45="","",$B$45)</f>
         <v/>
       </c>
       <c r="C63" s="4" t="n"/>
@@ -1403,11 +1393,11 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>Villa 5</t>
+          <t>Villa 4</t>
         </is>
       </c>
       <c r="B64" s="2">
-        <f>IF($B$47="","",$B$47)</f>
+        <f>IF($B$46="","",$B$46)</f>
         <v/>
       </c>
       <c r="C64" s="4" t="n"/>
@@ -1428,228 +1418,298 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
+          <t>Villa 5</t>
+        </is>
+      </c>
+      <c r="B65" s="2">
+        <f>IF($B$47="","",$B$47)</f>
+        <v/>
+      </c>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="3" t="n"/>
+      <c r="E65" s="10">
+        <f>$B$13*C65</f>
+        <v/>
+      </c>
+      <c r="F65" s="3">
+        <f>E65*D65</f>
+        <v/>
+      </c>
+      <c r="G65" s="5">
+        <f>F65*$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="n"/>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="11">
-        <f>SUM(E60:E64)</f>
-        <v/>
-      </c>
-      <c r="F65" s="9">
-        <f>SUM(F60:F64)</f>
-        <v/>
-      </c>
-      <c r="G65" s="8">
-        <f>SUM(G60:G64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t>Poste</t>
-        </is>
-      </c>
-      <c r="B67" s="1" t="inlineStr">
-        <is>
-          <t>Taux</t>
-        </is>
-      </c>
-      <c r="C67" s="1" t="inlineStr">
-        <is>
-          <t>Montant IDR</t>
-        </is>
-      </c>
-      <c r="D67" s="1" t="inlineStr">
-        <is>
-          <t>Montant EUR</t>
-        </is>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="11">
+        <f>SUM(E61:E65)</f>
+        <v/>
+      </c>
+      <c r="F66" s="9">
+        <f>SUM(F61:F65)</f>
+        <v/>
+      </c>
+      <c r="G66" s="8">
+        <f>SUM(G61:G65)</f>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>Taux</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="inlineStr">
+        <is>
+          <t>Montant IDR</t>
+        </is>
+      </c>
+      <c r="D68" s="1" t="inlineStr">
+        <is>
+          <t>Montant EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
           <t>REVENUS BRUTS ANNUELS</t>
         </is>
       </c>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="8">
-        <f>G65</f>
-        <v/>
-      </c>
-      <c r="D68" s="9">
-        <f>F65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="8">
+        <f>G66</f>
+        <v/>
+      </c>
+      <c r="D69" s="9">
+        <f>F66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Charges d'exploitation</t>
         </is>
       </c>
-      <c r="B69" s="4">
+      <c r="B70" s="4">
         <f>$B$57</f>
         <v/>
       </c>
-      <c r="C69" s="5">
-        <f>C68*$B$57</f>
-        <v/>
-      </c>
-      <c r="D69" s="3">
-        <f>C69/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="inlineStr">
+      <c r="C70" s="5">
+        <f>C69*$B$57</f>
+        <v/>
+      </c>
+      <c r="D70" s="3">
+        <f>C70/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Impôt sur les sociétés (sur le chiffre d'affaires)</t>
+        </is>
+      </c>
+      <c r="B71" s="4">
+        <f>$B$58</f>
+        <v/>
+      </c>
+      <c r="C71" s="5">
+        <f>C69*$B$58</f>
+        <v/>
+      </c>
+      <c r="D71" s="3">
+        <f>C71/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL DES CHARGES</t>
+        </is>
+      </c>
+      <c r="B72" s="4">
+        <f>IF(C69=0,0,C72/C69)</f>
+        <v/>
+      </c>
+      <c r="C72" s="5">
+        <f>C70+C71</f>
+        <v/>
+      </c>
+      <c r="D72" s="3">
+        <f>C72/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
         <is>
           <t>REVENUS NETS ANNUELS</t>
         </is>
       </c>
-      <c r="B70" s="7" t="n"/>
-      <c r="C70" s="8">
-        <f>C68-C69</f>
-        <v/>
-      </c>
-      <c r="D70" s="9">
-        <f>C70/$B$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="1" t="inlineStr">
+      <c r="B73" s="7" t="n"/>
+      <c r="C73" s="8">
+        <f>C69-C72</f>
+        <v/>
+      </c>
+      <c r="D73" s="9">
+        <f>C73/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
         <is>
           <t>INDICATEURS</t>
         </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Nombre de villas retenues dans le scénario</t>
-        </is>
-      </c>
-      <c r="B73" s="8">
-        <f>COUNTIF(D60:D64,"&gt;0")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>Rendement brut (revenus bruts / investissement total)</t>
-        </is>
-      </c>
-      <c r="B74" s="7">
-        <f>IF(C54=0,0,C68/C54)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>Rendement net (revenus nets / investissement total)</t>
-        </is>
-      </c>
-      <c r="B75" s="7">
-        <f>IF(C54=0,0,C70/C54)</f>
-        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Retour sur investissement (années)</t>
-        </is>
-      </c>
-      <c r="B76" s="11">
-        <f>IF(C70=0,0,C54/C70)</f>
+          <t>Nombre de villas retenues dans le scénario</t>
+        </is>
+      </c>
+      <c r="B76" s="8">
+        <f>COUNTIF(D61:D65,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Rendement brut (revenus bruts / investissement total)</t>
+        </is>
+      </c>
+      <c r="B77" s="7">
+        <f>IF(C54=0,0,C69/C54)</f>
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="inlineStr">
-        <is>
-          <t>NOTES / HYPOTHESES</t>
-        </is>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Rendement net (revenus nets / investissement total)</t>
+        </is>
+      </c>
+      <c r="B78" s="7">
+        <f>IF(C54=0,0,C73/C54)</f>
+        <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>MODE D'EMPLOI : renseigner le terrain (tableau 1), nommer les villas et saisir leurs budgets (tableau 2), puis leur occupation et leur prix de nuitee (tableau 3). Les villas non utilisees restent vides et comptent pour zero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>Tableau 1 : le choix FREEHOLD / LEASEHOLD en B16 pilote le calcul du prix du terrain ; le prix inutilise est simplement ignore. 1 are = 100 m2.</t>
-        </is>
+          <t>Retour sur investissement (années)</t>
+        </is>
+      </c>
+      <c r="B79" s="11">
+        <f>IF(C73=0,0,C54/C73)</f>
+        <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>Les prix du terrain sont des PRIX VENDEUR : la commission agence est ajoutee separement en ligne 29, uniquement si B22 = OUI, au taux de la cellule B23.</t>
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>NOTES / HYPOTHESES</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 30) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
+          <t>MODE D'EMPLOI : renseigner le terrain (tableau 1), nommer les villas et saisir leurs budgets (tableau 2), puis leur occupation et leur prix de nuitee (tableau 3). Les villas non utilisees restent vides et comptent pour zero.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>S'ajoutent au cout foncier le geometre (B11), les frais d'emmenagement (B24) et la ceremonie traditionnelle (B25), saisis en IDR.</t>
+          <t>Tableau 1 : le choix FREEHOLD / LEASEHOLD en B16 pilote le calcul du prix du terrain ; le prix inutilise est simplement ignore. 1 are = 100 m2.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Tableau 2 : une ligne par villa, construction et ameublement saisis en EUR ; pour un devis en IDR, saisir =montant_IDR/$B$7. La designation saisie en colonne B est reprise automatiquement dans le tableau 3.</t>
+          <t>Les prix du terrain sont des PRIX VENDEUR : la commission agence est ajoutee separement en ligne 29, uniquement si B22 = OUI, au taux de la cellule B23.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B40 = OUI, quel que soit le nombre de villas.</t>
+          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 30) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Tableau 3 : chaque villa a son propre taux d'occupation et son propre prix de nuitee. Revenus bruts = nuits commercialisables (B13) x taux d'occupation x prix de la nuitee. Les charges s'appliquent au revenu brut cumule.</t>
+          <t>S'ajoutent au cout foncier le geometre (B11), les frais d'emmenagement (B24) et la ceremonie traditionnelle (B25), saisis en IDR.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Taux de change en B7 : reference BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). A actualiser avant presentation au client.</t>
+          <t>Tableau 2 : une ligne par villa, construction et ameublement saisis en EUR ; pour un devis en IDR, saisir =montant_IDR/$B$7. La designation saisie en colonne B est reprise automatiquement dans le tableau 3.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Projection previsionnelle a but indicatif : elle n'integre ni la fiscalite indonesienne sur les revenus locatifs, ni l'amortissement, ni les frais de gestion au-dela du pourcentage de charges saisi. En leasehold, le rendement doit s'apprecier au regard de la duree residuelle du bail.</t>
+          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B40 = OUI, quel que soit le nombre de villas.</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="inlineStr">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Tableau 3 : chaque villa a son propre taux d'occupation et son propre prix de nuitée. Revenus bruts = nuits commercialisables (B13) x taux d'occupation x prix de la nuitée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Les charges regroupent les charges d'exploitation (B57) et l'impôt sur les sociétés (B58), ce dernier assis sur le chiffre d'affaires brut et non sur le résultat : il reste dû même sans bénéfice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Taux de change en B7 : référence BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). À actualiser avant présentation au client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Projection prévisionnelle à but indicatif : hors impôt sur les sociétés assis sur le chiffre d'affaires, elle n'intègre aucune autre fiscalité, ni l'amortissement, ni les frais de gestion au-delà du pourcentage de charges saisi. En leasehold, le rendement doit s'apprécier au regard de la durée résiduelle du bail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr">
         <is>
           <t>VERSION INTERNE - contient la commission agence. Ne pas transmettre au client : utiliser la version 'presentation client'.</t>
         </is>

</xml_diff>

<commit_message>
Version client : frais d'agence en montant désigné, sans pourcentage
Le tableau client affiche désormais le prix du terrain puis une ligne 'Frais
d'agence' à saisir manuellement, sans aucun taux, et leur sous-total sert de
base aux frais de notaire. Sa structure reflète celle de la version interne
(prix vendeur + commission), si bien que les deux fichiers aboutissent au même
coût foncier une fois le montant de commission reporté.

Les cellules de prix du tableau client attendent en conséquence le prix
vendeur, la commission n'y étant plus incorporée : elle serait sinon comptée
deux fois. Les notes internes rappellent la marche à suivre pour le report.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Projection_de_projet.xlsx
+++ b/transactions/Projection_de_projet.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1648,68 +1648,75 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Les prix du terrain sont des PRIX VENDEUR : la commission agence est ajoutee separement en ligne 29, uniquement si B22 = OUI, au taux de la cellule B23.</t>
+          <t>Les prix du terrain sont des PRIX VENDEUR : la commission agence est ajoutée séparément en ligne 29, uniquement si B22 = OUI, au taux de la cellule B23.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 30) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
+          <t>REPORT VERS LE TABLEAU CLIENT : ajuster le taux de commission jusqu'au montant voulu, puis reporter le montant de la ligne 29 dans la ligne 'Frais d'agence' du tableau client. Ce dernier attend le PRIX VENDEUR dans ses cellules de prix : la commission n'y est comptée qu'une fois, en frais d'agence.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>S'ajoutent au cout foncier le geometre (B11), les frais d'emmenagement (B24) et la ceremonie traditionnelle (B25), saisis en IDR.</t>
+          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 30) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Tableau 2 : une ligne par villa, construction et ameublement saisis en EUR ; pour un devis en IDR, saisir =montant_IDR/$B$7. La designation saisie en colonne B est reprise automatiquement dans le tableau 3.</t>
+          <t>S'ajoutent au cout foncier le geometre (B11), les frais d'emmenagement (B24) et la ceremonie traditionnelle (B25), saisis en IDR.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B40 = OUI, quel que soit le nombre de villas.</t>
+          <t>Tableau 2 : une ligne par villa, construction et ameublement saisis en EUR ; pour un devis en IDR, saisir =montant_IDR/$B$7. La designation saisie en colonne B est reprise automatiquement dans le tableau 3.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Tableau 3 : chaque villa a son propre taux d'occupation et son propre prix de nuitée. Revenus bruts = nuits commercialisables (B13) x taux d'occupation x prix de la nuitée.</t>
+          <t>La creation de la PT PMA (2 000 EUR, cellule B12) s'ajoute a l'investissement uniquement si B40 = OUI, quel que soit le nombre de villas.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Les charges regroupent les charges d'exploitation (B57) et l'impôt sur les sociétés (B58), ce dernier assis sur le chiffre d'affaires brut et non sur le résultat : il reste dû même sans bénéfice.</t>
+          <t>Tableau 3 : chaque villa a son propre taux d'occupation et son propre prix de nuitée. Revenus bruts = nuits commercialisables (B13) x taux d'occupation x prix de la nuitée.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Taux de change en B7 : référence BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). À actualiser avant présentation au client.</t>
+          <t>Les charges regroupent les charges d'exploitation (B57) et l'impôt sur les sociétés (B58), ce dernier assis sur le chiffre d'affaires brut et non sur le résultat : il reste dû même sans bénéfice.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
+          <t>Taux de change en B7 : référence BCE du 20/08/2026 (1 EUR = 20 788,62 IDR). À actualiser avant présentation au client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
           <t>Projection prévisionnelle à but indicatif : hors impôt sur les sociétés assis sur le chiffre d'affaires, elle n'intègre aucune autre fiscalité, ni l'amortissement, ni les frais de gestion au-delà du pourcentage de charges saisi. En leasehold, le rendement doit s'apprécier au regard de la durée résiduelle du bail.</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="1" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
         <is>
           <t>VERSION INTERNE - contient la commission agence. Ne pas transmettre au client : utiliser la version 'presentation client'.</t>
         </is>

</xml_diff>

<commit_message>
Assied les frais de notaire sur le prix officiel du terrain
Taxes gouvernementales et honoraires du notaire portent desormais sur le prix
vendeur declare a l'acte, commission ou frais d'agence exclus, dans les quatre
tableaux : projection interne, projection client et les deux recapitulatifs
d'appel de fonds. Les libelles et les notes le precisent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Projection_de_projet.xlsx
+++ b/transactions/Projection_de_projet.xlsx
@@ -882,7 +882,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Taxes gouvernementales</t>
+          <t>Taxes gouvernementales (sur le prix officiel du terrain)</t>
         </is>
       </c>
       <c r="B31" s="4">
@@ -890,7 +890,7 @@
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>C30*$B$8</f>
+        <f>C28*$B$8</f>
         <v/>
       </c>
       <c r="D31" s="3">
@@ -901,15 +901,15 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire (forfait plancher en B10)</t>
+          <t>Honoraires du notaire (sur le prix officiel, forfait plancher en B10)</t>
         </is>
       </c>
       <c r="B32" s="4">
-        <f>IF(C30=0,0,C32/C30)</f>
+        <f>IF(C28=0,0,C32/C28)</f>
         <v/>
       </c>
       <c r="C32" s="5">
-        <f>MAX(C30*$B$9,$B$10)</f>
+        <f>MAX(C28*$B$9,$B$10)</f>
         <v/>
       </c>
       <c r="D32" s="3">
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="B33" s="4">
-        <f>IF(C30=0,0,C33/C30)</f>
+        <f>IF(C28=0,0,C33/C28)</f>
         <v/>
       </c>
       <c r="C33" s="5">
@@ -1662,7 +1662,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Les frais de notaire portent sur le prix du terrain commission comprise (ligne 30) : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
+          <t>Les frais de notaire portent sur le PRIX OFFICIEL du terrain (ligne 28), commission exclue : taxes gouvernementales (B8) + honoraires (B9) avec un forfait plancher de 20 000 000 IDR (B10).</t>
         </is>
       </c>
     </row>

</xml_diff>